<commit_message>
25/3/26 import new produk
</commit_message>
<xml_diff>
--- a/public/dokumen/template-import-produk.xlsx
+++ b/public/dokumen/template-import-produk.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K89"/>
+  <dimension ref="A1:K69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -476,38 +476,38 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ANCAMIDE 261A</t>
+          <t>Epoxy - Kaleng 1 kg</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Umum</t>
+          <t>EPOXY</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>100022</t>
+          <t>k - 1</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>Set</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="F2" t="n">
         <v>1</v>
       </c>
       <c r="G2" t="n">
-        <v>1488000</v>
+        <v>107000</v>
       </c>
       <c r="H2" t="n">
-        <v>0</v>
+        <v>1284000</v>
       </c>
       <c r="I2" t="n">
-        <v>0</v>
+        <v>107000</v>
       </c>
       <c r="J2" t="n">
         <v>0</v>
@@ -517,38 +517,38 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Alifatik Lem DN 20 KG</t>
+          <t>Epoxy - Kaleng 1/2 kg</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Lem DN</t>
+          <t>EPOXY</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>DN20</t>
+          <t>k - 1/2</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>PCS</t>
+          <t>Set</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>1</v>
+        <v>24</v>
       </c>
       <c r="F3" t="n">
         <v>1</v>
       </c>
       <c r="G3" t="n">
-        <v>360000</v>
+        <v>54000</v>
       </c>
       <c r="H3" t="n">
-        <v>0</v>
+        <v>1296000</v>
       </c>
       <c r="I3" t="n">
-        <v>0</v>
+        <v>54000</v>
       </c>
       <c r="J3" t="n">
         <v>0</v>
@@ -558,38 +558,38 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Alifatik Lem DN 3,5 KG</t>
+          <t>Epoxy - Kaleng 1/4 kg</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Umum</t>
+          <t>EPOXY</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>DN35KG</t>
+          <t>k - 1/4</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>PCS</t>
+          <t>Set</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>1</v>
+        <v>48</v>
       </c>
       <c r="F4" t="n">
         <v>1</v>
       </c>
       <c r="G4" t="n">
-        <v>80000</v>
+        <v>32000</v>
       </c>
       <c r="H4" t="n">
-        <v>0</v>
+        <v>1536000</v>
       </c>
       <c r="I4" t="n">
-        <v>0</v>
+        <v>32000</v>
       </c>
       <c r="J4" t="n">
         <v>0</v>
@@ -599,38 +599,38 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Alifatik Lem DN 4KG</t>
+          <t>Epoxy Botol 1 kg</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Umum</t>
+          <t>EPOXY</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>DN4</t>
+          <t>b - 1</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>PCS</t>
+          <t>Set</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F5" t="n">
         <v>1</v>
       </c>
       <c r="G5" t="n">
-        <v>90000</v>
+        <v>124000</v>
       </c>
       <c r="H5" t="n">
-        <v>0</v>
+        <v>1240000</v>
       </c>
       <c r="I5" t="n">
-        <v>0</v>
+        <v>124000</v>
       </c>
       <c r="J5" t="n">
         <v>0</v>
@@ -640,38 +640,38 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Alifatik Lem DN 600ml</t>
+          <t>Epoxy - Botol 1/2 kg</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Lem DN</t>
+          <t>EPOXY</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>DN600</t>
+          <t>b- 1/2</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>PCS</t>
+          <t>Set</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="F6" t="n">
         <v>1</v>
       </c>
       <c r="G6" t="n">
-        <v>17500</v>
+        <v>68000</v>
       </c>
       <c r="H6" t="n">
-        <v>0</v>
+        <v>1020000</v>
       </c>
       <c r="I6" t="n">
-        <v>0</v>
+        <v>68000</v>
       </c>
       <c r="J6" t="n">
         <v>0</v>
@@ -681,17 +681,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>B1Kg Resin</t>
+          <t>Epoxy - Botol 1/4 kg</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>epoxy</t>
+          <t>EPOXY</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>B1R</t>
+          <t>b - 1/4</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -700,19 +700,19 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>1</v>
+        <v>48</v>
       </c>
       <c r="F7" t="n">
         <v>1</v>
       </c>
       <c r="G7" t="n">
-        <v>86500</v>
+        <v>31000</v>
       </c>
       <c r="H7" t="n">
-        <v>0</v>
+        <v>1488000</v>
       </c>
       <c r="I7" t="n">
-        <v>0</v>
+        <v>31000</v>
       </c>
       <c r="J7" t="n">
         <v>0</v>
@@ -722,38 +722,38 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>BE188</t>
+          <t>Epoxy New - Kaleng 1 kg</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Umum</t>
+          <t>EPOXY</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>100019</t>
+          <t>K - 1 New</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Drum</t>
+          <t>Set</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="F8" t="n">
         <v>1</v>
       </c>
       <c r="G8" t="n">
-        <v>78650</v>
+        <v>99000</v>
       </c>
       <c r="H8" t="n">
-        <v>0</v>
+        <v>1188000</v>
       </c>
       <c r="I8" t="n">
-        <v>0</v>
+        <v>99000</v>
       </c>
       <c r="J8" t="n">
         <v>0</v>
@@ -763,17 +763,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Botol Clear Epoxy  1KG</t>
+          <t>Epoxy New - Botol 1 kg</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>EPOXY CLEAR</t>
+          <t>EPOXY</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>100084</t>
+          <t>B - 1 New</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -782,19 +782,19 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F9" t="n">
         <v>1</v>
       </c>
       <c r="G9" t="n">
-        <v>108000</v>
+        <v>107000</v>
       </c>
       <c r="H9" t="n">
-        <v>0</v>
+        <v>1070000</v>
       </c>
       <c r="I9" t="n">
-        <v>0</v>
+        <v>107000</v>
       </c>
       <c r="J9" t="n">
         <v>0</v>
@@ -804,17 +804,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Botol Clear Epoxy 1/2KG</t>
+          <t>Epoxy New - Botol 1/2 kg</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>EPOXY CLEAR</t>
+          <t>EPOXY</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>100085</t>
+          <t>B - 1/2 New</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -823,7 +823,7 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="F10" t="n">
         <v>1</v>
@@ -832,10 +832,10 @@
         <v>54000</v>
       </c>
       <c r="H10" t="n">
-        <v>0</v>
+        <v>810000</v>
       </c>
       <c r="I10" t="n">
-        <v>0</v>
+        <v>54000</v>
       </c>
       <c r="J10" t="n">
         <v>0</v>
@@ -845,17 +845,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Botol Clear Epoxy 1/4KG</t>
+          <t>EPOXY Wood Lux - Botol R 06 H 07 1 kg</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>EPOXY CLEAR</t>
+          <t>EPOXY</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>100086</t>
+          <t>B - 1 WL</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -864,19 +864,19 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F11" t="n">
         <v>1</v>
       </c>
       <c r="G11" t="n">
-        <v>30000</v>
+        <v>85000</v>
       </c>
       <c r="H11" t="n">
-        <v>0</v>
+        <v>850000</v>
       </c>
       <c r="I11" t="n">
-        <v>0</v>
+        <v>85000</v>
       </c>
       <c r="J11" t="n">
         <v>0</v>
@@ -886,17 +886,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Botol Polos 1 Kg</t>
+          <t>EPOXY Wood Lux - Botol R 03 H 035 1/2 kg</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Polos</t>
+          <t>EPOXY</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>BP1</t>
+          <t>B - 1/2 WL</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -905,19 +905,19 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F12" t="n">
         <v>1</v>
       </c>
       <c r="G12" t="n">
-        <v>94000</v>
+        <v>45000</v>
       </c>
       <c r="H12" t="n">
-        <v>0</v>
+        <v>675000</v>
       </c>
       <c r="I12" t="n">
-        <v>0</v>
+        <v>45000</v>
       </c>
       <c r="J12" t="n">
         <v>0</v>
@@ -927,17 +927,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Botol Polos 1/2 Kg</t>
+          <t>EPOXY Polos - Botol RH 07 1 kg</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Polos</t>
+          <t>EPOXY</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>BP1/2</t>
+          <t>B - 1P</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -946,19 +946,19 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="F13" t="n">
         <v>1</v>
       </c>
       <c r="G13" t="n">
-        <v>49500</v>
+        <v>97000</v>
       </c>
       <c r="H13" t="n">
-        <v>0</v>
+        <v>970000</v>
       </c>
       <c r="I13" t="n">
-        <v>0</v>
+        <v>97000</v>
       </c>
       <c r="J13" t="n">
         <v>0</v>
@@ -968,38 +968,38 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Customize</t>
+          <t>EPOXY Polos - Botol RH 035 1/2 kg</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>DRUM</t>
+          <t>EPOXY</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>100021</t>
+          <t>B - 1/2 P</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Drum</t>
+          <t>Set</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="F14" t="n">
         <v>1</v>
       </c>
       <c r="G14" t="n">
-        <v>0</v>
+        <v>51000</v>
       </c>
       <c r="H14" t="n">
-        <v>0</v>
+        <v>765000</v>
       </c>
       <c r="I14" t="n">
-        <v>0</v>
+        <v>51000</v>
       </c>
       <c r="J14" t="n">
         <v>0</v>
@@ -1009,17 +1009,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>EPOXY B1/2kg WoodLux</t>
+          <t>Epoxy - Pill 20 kg</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>epoxy</t>
+          <t>EPOXY</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>WLB1/2</t>
+          <t>P - 20</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1028,19 +1028,19 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="F15" t="n">
         <v>1</v>
       </c>
       <c r="G15" t="n">
-        <v>45000</v>
+        <v>2850000</v>
       </c>
       <c r="H15" t="n">
-        <v>0</v>
+        <v>2850000</v>
       </c>
       <c r="I15" t="n">
-        <v>0</v>
+        <v>2850000</v>
       </c>
       <c r="J15" t="n">
         <v>0</v>
@@ -1050,17 +1050,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>EPOXY B1Kg WoodLux</t>
+          <t>Epoxy - Pill 18 kg</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Umum</t>
+          <t>EPOXY</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>WLB1</t>
+          <t>P - 18</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1069,19 +1069,19 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="F16" t="n">
         <v>1</v>
       </c>
       <c r="G16" t="n">
-        <v>85000</v>
+        <v>2572000</v>
       </c>
       <c r="H16" t="n">
-        <v>0</v>
+        <v>2572000</v>
       </c>
       <c r="I16" t="n">
-        <v>0</v>
+        <v>2572000</v>
       </c>
       <c r="J16" t="n">
         <v>0</v>
@@ -1091,17 +1091,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>EPOXY Jerigen 4Kg</t>
+          <t>Epoxy - Pill 16 kg</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>epoxy</t>
+          <t>EPOXY</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>J4</t>
+          <t>P - 16</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1116,13 +1116,13 @@
         <v>1</v>
       </c>
       <c r="G17" t="n">
-        <v>572000</v>
+        <v>2298000</v>
       </c>
       <c r="H17" t="n">
-        <v>0</v>
+        <v>2298000</v>
       </c>
       <c r="I17" t="n">
-        <v>0</v>
+        <v>2298000</v>
       </c>
       <c r="J17" t="n">
         <v>0</v>
@@ -1132,17 +1132,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>EPOXY Jerigen 5Kg</t>
+          <t>Epoxy - Jerigen 5 kg</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>MR LUX Jerigen</t>
+          <t>EPOXY</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>J5</t>
+          <t>J - 5</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1160,10 +1160,10 @@
         <v>716500</v>
       </c>
       <c r="H18" t="n">
-        <v>0</v>
+        <v>716500</v>
       </c>
       <c r="I18" t="n">
-        <v>0</v>
+        <v>716500</v>
       </c>
       <c r="J18" t="n">
         <v>0</v>
@@ -1173,17 +1173,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>EPOXY Pail 16 KG</t>
+          <t>Epoxy - Jerigen 4 kg</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Umum</t>
+          <t>EPOXY</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>100068</t>
+          <t>J - 4</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1198,13 +1198,13 @@
         <v>1</v>
       </c>
       <c r="G19" t="n">
-        <v>2298000</v>
+        <v>572000</v>
       </c>
       <c r="H19" t="n">
-        <v>0</v>
+        <v>572000</v>
       </c>
       <c r="I19" t="n">
-        <v>0</v>
+        <v>572000</v>
       </c>
       <c r="J19" t="n">
         <v>0</v>
@@ -1214,19 +1214,15 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>EPOXY Pail 18 KG</t>
+          <t>Telp.(024) 7624836 / +62818452014</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Umum</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>100069</t>
-        </is>
-      </c>
+          <t>EPOXY</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr">
         <is>
           <t>Set</t>
@@ -1239,7 +1235,7 @@
         <v>1</v>
       </c>
       <c r="G20" t="n">
-        <v>2572000</v>
+        <v>0</v>
       </c>
       <c r="H20" t="n">
         <v>0</v>
@@ -1255,19 +1251,15 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>EPOXY Pail 20 KG</t>
+          <t>Website : https://mrluxindonesia.com/</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Umum</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>100070</t>
-        </is>
-      </c>
+          <t>EPOXY</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr">
         <is>
           <t>Set</t>
@@ -1280,7 +1272,7 @@
         <v>1</v>
       </c>
       <c r="G21" t="n">
-        <v>2850000</v>
+        <v>0</v>
       </c>
       <c r="H21" t="n">
         <v>0</v>
@@ -1296,19 +1288,15 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Epoxy Kaleng 1 Kg</t>
+          <t>EPOXY</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Umum</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>100001</t>
-        </is>
-      </c>
+          <t>EPOXY</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr">
         <is>
           <t>Set</t>
@@ -1321,7 +1309,7 @@
         <v>1</v>
       </c>
       <c r="G22" t="n">
-        <v>110819</v>
+        <v>0</v>
       </c>
       <c r="H22" t="n">
         <v>0</v>
@@ -1337,22 +1325,22 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>HARDENER ACR</t>
+          <t>NAMA BARANG PACKAGING QTY</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>DRUM</t>
+          <t>EPOXY</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>100075</t>
+          <t>CODE</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Drum</t>
+          <t>Set</t>
         </is>
       </c>
       <c r="E23" t="n">
@@ -1378,38 +1366,38 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>HARDENER AP</t>
+          <t>EPOXY MR Lux KALENG 1 KG</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>DRUM</t>
+          <t>EPOXY</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>100076</t>
+          <t>K - 1</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Drum</t>
+          <t>Set</t>
         </is>
       </c>
       <c r="E24" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="F24" t="n">
         <v>1</v>
       </c>
       <c r="G24" t="n">
-        <v>0</v>
+        <v>120000</v>
       </c>
       <c r="H24" t="n">
-        <v>0</v>
+        <v>1440000</v>
       </c>
       <c r="I24" t="n">
-        <v>0</v>
+        <v>120000</v>
       </c>
       <c r="J24" t="n">
         <v>0</v>
@@ -1419,38 +1407,38 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>HARDENER SUNMIDE</t>
+          <t>EPOXY MR Lux KALENG 1/2 KG</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>DRUM</t>
+          <t>EPOXY</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>100077</t>
+          <t>K - 1/2</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Drum</t>
+          <t>Set</t>
         </is>
       </c>
       <c r="E25" t="n">
-        <v>1</v>
+        <v>24</v>
       </c>
       <c r="F25" t="n">
         <v>1</v>
       </c>
       <c r="G25" t="n">
-        <v>0</v>
+        <v>60500</v>
       </c>
       <c r="H25" t="n">
-        <v>0</v>
+        <v>1452000</v>
       </c>
       <c r="I25" t="n">
-        <v>0</v>
+        <v>60500</v>
       </c>
       <c r="J25" t="n">
         <v>0</v>
@@ -1460,38 +1448,38 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Hardener</t>
+          <t>EPOXY MR Lux KALENG 1/4 KG</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>epoxy</t>
+          <t>EPOXY</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>100017</t>
+          <t>K - 1/4</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>Set</t>
         </is>
       </c>
       <c r="E26" t="n">
-        <v>1</v>
+        <v>48</v>
       </c>
       <c r="F26" t="n">
         <v>1</v>
       </c>
       <c r="G26" t="n">
-        <v>0</v>
+        <v>36000</v>
       </c>
       <c r="H26" t="n">
-        <v>0</v>
+        <v>1728000</v>
       </c>
       <c r="I26" t="n">
-        <v>0</v>
+        <v>36000</v>
       </c>
       <c r="J26" t="n">
         <v>0</v>
@@ -1501,17 +1489,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Jerigen 5kg</t>
+          <t>EPOXY MR Lux BOTOL 1 KG</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Umum</t>
+          <t>EPOXY</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>100043</t>
+          <t>B - 1</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1520,19 +1508,19 @@
         </is>
       </c>
       <c r="E27" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F27" t="n">
         <v>1</v>
       </c>
       <c r="G27" t="n">
-        <v>716500</v>
+        <v>138500</v>
       </c>
       <c r="H27" t="n">
-        <v>0</v>
+        <v>1385000</v>
       </c>
       <c r="I27" t="n">
-        <v>0</v>
+        <v>138500</v>
       </c>
       <c r="J27" t="n">
         <v>0</v>
@@ -1542,38 +1530,38 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>KREOLIN TUTUP DOBEL  PRINTING</t>
+          <t>EPOXY MR Lux BOTOL 1/2 KG</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>BOTOL KOSONG</t>
+          <t>EPOXY</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>KR1MR</t>
+          <t>B - 1/2</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>PCS</t>
+          <t>Set</t>
         </is>
       </c>
       <c r="E28" t="n">
-        <v>50</v>
+        <v>15</v>
       </c>
       <c r="F28" t="n">
         <v>1</v>
       </c>
       <c r="G28" t="n">
-        <v>0</v>
+        <v>76000</v>
       </c>
       <c r="H28" t="n">
-        <v>0</v>
+        <v>1140000</v>
       </c>
       <c r="I28" t="n">
-        <v>0</v>
+        <v>76000</v>
       </c>
       <c r="J28" t="n">
         <v>0</v>
@@ -1583,38 +1571,38 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>KUKDO G0930</t>
+          <t>EPOXY MR Lux BOTOL 1/4 KG</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Umum</t>
+          <t>EPOXY</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>100023</t>
+          <t>B - 1/4</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>Set</t>
         </is>
       </c>
       <c r="E29" t="n">
-        <v>1</v>
+        <v>48</v>
       </c>
       <c r="F29" t="n">
         <v>1</v>
       </c>
       <c r="G29" t="n">
-        <v>1536000</v>
+        <v>35000</v>
       </c>
       <c r="H29" t="n">
-        <v>0</v>
+        <v>1680000</v>
       </c>
       <c r="I29" t="n">
-        <v>0</v>
+        <v>35000</v>
       </c>
       <c r="J29" t="n">
         <v>0</v>
@@ -1624,38 +1612,38 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Lem Alteco HQ</t>
+          <t>EPOXY New MR Lux BOTOL 1 KG</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>HQ</t>
+          <t>EPOXY</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>HQ</t>
+          <t>B - 1 N</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>PCS</t>
+          <t>Set</t>
         </is>
       </c>
       <c r="E30" t="n">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="F30" t="n">
         <v>1</v>
       </c>
       <c r="G30" t="n">
-        <v>3400</v>
+        <v>120000</v>
       </c>
       <c r="H30" t="n">
-        <v>0</v>
+        <v>1200000</v>
       </c>
       <c r="I30" t="n">
-        <v>0</v>
+        <v>120000</v>
       </c>
       <c r="J30" t="n">
         <v>0</v>
@@ -1665,38 +1653,38 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Lem Cair MR lUX (CYANOACRYLATE)</t>
+          <t>EPOXY New MR Lux BOTOL 1/2 KG</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>HQ</t>
+          <t>EPOXY</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>100081</t>
+          <t>B - 1/2 N</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>PCS</t>
+          <t>Set</t>
         </is>
       </c>
       <c r="E31" t="n">
-        <v>50</v>
+        <v>15</v>
       </c>
       <c r="F31" t="n">
         <v>1</v>
       </c>
       <c r="G31" t="n">
-        <v>6250</v>
+        <v>60500</v>
       </c>
       <c r="H31" t="n">
-        <v>0</v>
+        <v>907500</v>
       </c>
       <c r="I31" t="n">
-        <v>0</v>
+        <v>60500</v>
       </c>
       <c r="J31" t="n">
         <v>0</v>
@@ -1706,22 +1694,18 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Lem PU adhesive</t>
+          <t>POLYURETHANE (PU)</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Umum</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>100047</t>
-        </is>
-      </c>
+          <t>EPOXY</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr"/>
       <c r="D32" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>Set</t>
         </is>
       </c>
       <c r="E32" t="n">
@@ -1747,38 +1731,38 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Lem Putih S30(H)</t>
+          <t>PU MR Lux BOTOL 1 KG</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Lem Putih</t>
+          <t>EPOXY</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>S30</t>
+          <t>PU - 1 MR Lux</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>PCS</t>
+          <t>Set</t>
         </is>
       </c>
       <c r="E33" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="F33" t="n">
         <v>1</v>
       </c>
       <c r="G33" t="n">
-        <v>1000</v>
+        <v>69000</v>
       </c>
       <c r="H33" t="n">
-        <v>0</v>
+        <v>1380000</v>
       </c>
       <c r="I33" t="n">
-        <v>0</v>
+        <v>69000</v>
       </c>
       <c r="J33" t="n">
         <v>0</v>
@@ -1788,38 +1772,38 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Lem Putih S30(H) 2,5 kg</t>
+          <t>PU MR Lux BOTOL 1/2 KG</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Lem Putih</t>
+          <t>EPOXY</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>100062</t>
+          <t>PU- 1/2 MR Lux</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>PCS</t>
+          <t>Set</t>
         </is>
       </c>
       <c r="E34" t="n">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="F34" t="n">
         <v>1</v>
       </c>
       <c r="G34" t="n">
-        <v>38000</v>
+        <v>35500</v>
       </c>
       <c r="H34" t="n">
-        <v>0</v>
+        <v>1065000</v>
       </c>
       <c r="I34" t="n">
-        <v>0</v>
+        <v>35500</v>
       </c>
       <c r="J34" t="n">
         <v>0</v>
@@ -1829,38 +1813,38 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Lem Putih S30(H) 3,5 ons</t>
+          <t>PU MR Lux BOTOL 1/4 KG</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Lem Putih</t>
+          <t>EPOXY</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>H350</t>
+          <t>PU- 1/4 MR Lux</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>PCS</t>
+          <t>Set</t>
         </is>
       </c>
       <c r="E35" t="n">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="F35" t="n">
         <v>1</v>
       </c>
       <c r="G35" t="n">
-        <v>5500</v>
+        <v>17000</v>
       </c>
       <c r="H35" t="n">
-        <v>0</v>
+        <v>1632000</v>
       </c>
       <c r="I35" t="n">
-        <v>0</v>
+        <v>17000</v>
       </c>
       <c r="J35" t="n">
         <v>0</v>
@@ -1870,38 +1854,38 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Lem Putih S30(H) 4 ons</t>
+          <t>PU MR Lux Putih/WL BOTOL 1 KG</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Lem Putih</t>
+          <t>EPOXY</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>H400</t>
+          <t>PU - 1 P</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>PCS</t>
+          <t>Set</t>
         </is>
       </c>
       <c r="E36" t="n">
-        <v>100</v>
+        <v>20</v>
       </c>
       <c r="F36" t="n">
         <v>1</v>
       </c>
       <c r="G36" t="n">
-        <v>6350</v>
+        <v>56000</v>
       </c>
       <c r="H36" t="n">
-        <v>0</v>
+        <v>1120000</v>
       </c>
       <c r="I36" t="n">
-        <v>0</v>
+        <v>56000</v>
       </c>
       <c r="J36" t="n">
         <v>0</v>
@@ -1911,38 +1895,38 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Lem Putih S30(H) 6,5 ons</t>
+          <t>PU MR Lux Putih/WL BOTOL 1/2 KG</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Lem Putih</t>
+          <t>EPOXY</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>H650</t>
+          <t>PU - 1/2 P</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>PCS</t>
+          <t>Set</t>
         </is>
       </c>
       <c r="E37" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="F37" t="n">
         <v>1</v>
       </c>
       <c r="G37" t="n">
-        <v>10200</v>
+        <v>27000</v>
       </c>
       <c r="H37" t="n">
-        <v>0</v>
+        <v>810000</v>
       </c>
       <c r="I37" t="n">
-        <v>0</v>
+        <v>27000</v>
       </c>
       <c r="J37" t="n">
         <v>0</v>
@@ -1952,38 +1936,38 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Lem Putih S30(H) 8 ons</t>
+          <t>PU MR Lux Putih/WL BOTOL 0.85 KG</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Lem Putih</t>
+          <t>EPOXY</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>H800</t>
+          <t>PU - 0.85</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>PCS</t>
+          <t>Set</t>
         </is>
       </c>
       <c r="E38" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="F38" t="n">
         <v>1</v>
       </c>
       <c r="G38" t="n">
-        <v>12250</v>
+        <v>53250</v>
       </c>
       <c r="H38" t="n">
-        <v>0</v>
+        <v>1065000</v>
       </c>
       <c r="I38" t="n">
-        <v>0</v>
+        <v>53250</v>
       </c>
       <c r="J38" t="n">
         <v>0</v>
@@ -1993,38 +1977,38 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Lem Putih S30(H) Gallon 3 kg</t>
+          <t>PU MR Lux Putih/WL BOTOL 0.8 KG</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Lem Putih</t>
+          <t>EPOXY</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>100063</t>
+          <t>PU - 0.8</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>PCS</t>
+          <t>Set</t>
         </is>
       </c>
       <c r="E39" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="F39" t="n">
         <v>1</v>
       </c>
       <c r="G39" t="n">
-        <v>56000</v>
+        <v>50400</v>
       </c>
       <c r="H39" t="n">
-        <v>0</v>
+        <v>1008000</v>
       </c>
       <c r="I39" t="n">
-        <v>0</v>
+        <v>50400</v>
       </c>
       <c r="J39" t="n">
         <v>0</v>
@@ -2034,22 +2018,18 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Lem Putih S40 (M) 1 kg</t>
+          <t>NON SAG</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Lem Putih</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>100087</t>
-        </is>
-      </c>
+          <t>EPOXY</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr"/>
       <c r="D40" t="inlineStr">
         <is>
-          <t>PCS</t>
+          <t>Set</t>
         </is>
       </c>
       <c r="E40" t="n">
@@ -2059,7 +2039,7 @@
         <v>1</v>
       </c>
       <c r="G40" t="n">
-        <v>17000</v>
+        <v>0</v>
       </c>
       <c r="H40" t="n">
         <v>0</v>
@@ -2075,38 +2055,38 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Lem Putih S40(M)</t>
+          <t>Non Sag KALENG 1 KG</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Lem Putih</t>
+          <t>EPOXY</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>100045</t>
+          <t>NS - 1</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>PCS</t>
+          <t>Set</t>
         </is>
       </c>
       <c r="E41" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="F41" t="n">
         <v>1</v>
       </c>
       <c r="G41" t="n">
-        <v>1000</v>
+        <v>203000</v>
       </c>
       <c r="H41" t="n">
-        <v>0</v>
+        <v>1624000</v>
       </c>
       <c r="I41" t="n">
-        <v>0</v>
+        <v>203000</v>
       </c>
       <c r="J41" t="n">
         <v>0</v>
@@ -2116,38 +2096,38 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Lem Putih S40(M) 3,5 ons</t>
+          <t>Non Sag KALENG 1/2 KG</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Lem Putih</t>
+          <t>EPOXY</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>M350</t>
+          <t>NS - 1 /2</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>PCS</t>
+          <t>Set</t>
         </is>
       </c>
       <c r="E42" t="n">
-        <v>100</v>
+        <v>12</v>
       </c>
       <c r="F42" t="n">
         <v>1</v>
       </c>
       <c r="G42" t="n">
-        <v>6000</v>
+        <v>116000</v>
       </c>
       <c r="H42" t="n">
-        <v>0</v>
+        <v>1392000</v>
       </c>
       <c r="I42" t="n">
-        <v>0</v>
+        <v>116000</v>
       </c>
       <c r="J42" t="n">
         <v>0</v>
@@ -2157,38 +2137,38 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Lem Putih S40(M) 4 ons</t>
+          <t>Non Sag KALENG 1/4 KG</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Lem Putih</t>
+          <t>EPOXY</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>M400</t>
+          <t>NS - 1/4</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>PCS</t>
+          <t>Set</t>
         </is>
       </c>
       <c r="E43" t="n">
-        <v>100</v>
+        <v>36</v>
       </c>
       <c r="F43" t="n">
         <v>1</v>
       </c>
       <c r="G43" t="n">
-        <v>7000</v>
+        <v>57000</v>
       </c>
       <c r="H43" t="n">
-        <v>0</v>
+        <v>2052000</v>
       </c>
       <c r="I43" t="n">
-        <v>0</v>
+        <v>57000</v>
       </c>
       <c r="J43" t="n">
         <v>0</v>
@@ -2198,38 +2178,38 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Lem Putih S40(M) 5,5 ons</t>
+          <t>Non Sag KALENG 1 ONS</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Lem Putih</t>
+          <t>EPOXY</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>M550</t>
+          <t>NS - 1 Oz</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>PCS</t>
+          <t>Set</t>
         </is>
       </c>
       <c r="E44" t="n">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="F44" t="n">
         <v>1</v>
       </c>
       <c r="G44" t="n">
-        <v>9300</v>
+        <v>28000</v>
       </c>
       <c r="H44" t="n">
-        <v>0</v>
+        <v>1344000</v>
       </c>
       <c r="I44" t="n">
-        <v>0</v>
+        <v>28000</v>
       </c>
       <c r="J44" t="n">
         <v>0</v>
@@ -2239,38 +2219,38 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Lem Putih S40(M) 6,5 ons</t>
+          <t>Alifatik BOTOL 600 GR</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Lem Putih</t>
+          <t>EPOXY</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>M650</t>
+          <t>AL - 600</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>PCS</t>
+          <t>Set</t>
         </is>
       </c>
       <c r="E45" t="n">
-        <v>50</v>
+        <v>1</v>
       </c>
       <c r="F45" t="n">
         <v>1</v>
       </c>
       <c r="G45" t="n">
-        <v>11200</v>
+        <v>19500</v>
       </c>
       <c r="H45" t="n">
         <v>0</v>
       </c>
       <c r="I45" t="n">
-        <v>0</v>
+        <v>19500</v>
       </c>
       <c r="J45" t="n">
         <v>0</v>
@@ -2280,38 +2260,38 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Lem Putih S40(M) 8 ons</t>
+          <t>Alifatik GALON 3,5 KG</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Lem Putih</t>
+          <t>EPOXY</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>M800</t>
+          <t>AL - 3,5</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>PCS</t>
+          <t>Set</t>
         </is>
       </c>
       <c r="E46" t="n">
-        <v>50</v>
+        <v>1</v>
       </c>
       <c r="F46" t="n">
         <v>1</v>
       </c>
       <c r="G46" t="n">
-        <v>13750</v>
+        <v>89500</v>
       </c>
       <c r="H46" t="n">
         <v>0</v>
       </c>
       <c r="I46" t="n">
-        <v>0</v>
+        <v>89500</v>
       </c>
       <c r="J46" t="n">
         <v>0</v>
@@ -2321,38 +2301,38 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Lem Putih S50(E) 2,5 kg</t>
+          <t>Alifatik GALON 4 KG</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Lem Putih</t>
+          <t>EPOXY</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>100052</t>
+          <t>AL - 4</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>PCS</t>
+          <t>Set</t>
         </is>
       </c>
       <c r="E47" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="F47" t="n">
         <v>1</v>
       </c>
       <c r="G47" t="n">
-        <v>49500</v>
+        <v>104000</v>
       </c>
       <c r="H47" t="n">
         <v>0</v>
       </c>
       <c r="I47" t="n">
-        <v>0</v>
+        <v>104000</v>
       </c>
       <c r="J47" t="n">
         <v>0</v>
@@ -2362,38 +2342,38 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Lem Putih S50(E) 4 ons</t>
+          <t>Alteco Pcs 45 ML</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Lem Putih</t>
+          <t>EPOXY</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>E400</t>
+          <t>Alt - 50</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>PCS</t>
+          <t>Set</t>
         </is>
       </c>
       <c r="E48" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="F48" t="n">
         <v>1</v>
       </c>
       <c r="G48" t="n">
-        <v>8000</v>
+        <v>6250</v>
       </c>
       <c r="H48" t="n">
-        <v>0</v>
+        <v>312500</v>
       </c>
       <c r="I48" t="n">
-        <v>0</v>
+        <v>6250</v>
       </c>
       <c r="J48" t="n">
         <v>0</v>
@@ -2403,32 +2383,28 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Lem Putih S50(E) 6,5 ons</t>
+          <t>Notte : Sewaktu waktu Harga Berubah</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Lem Putih</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>S50</t>
-        </is>
-      </c>
+          <t>EPOXY</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr"/>
       <c r="D49" t="inlineStr">
         <is>
-          <t>PCS</t>
+          <t>Set</t>
         </is>
       </c>
       <c r="E49" t="n">
-        <v>100</v>
+        <v>1</v>
       </c>
       <c r="F49" t="n">
         <v>1</v>
       </c>
       <c r="G49" t="n">
-        <v>13000</v>
+        <v>0</v>
       </c>
       <c r="H49" t="n">
         <v>0</v>
@@ -2444,7 +2420,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Lem Putih S50(E) 6,5 ons</t>
+          <t>GP - 5505 - HV (S = 50 EMAS) 3,5 ONS</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2452,27 +2428,23 @@
           <t>Lem Putih</t>
         </is>
       </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>E650</t>
-        </is>
-      </c>
+      <c r="C50" t="inlineStr"/>
       <c r="D50" t="inlineStr">
         <is>
           <t>PCS</t>
         </is>
       </c>
       <c r="E50" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="F50" t="n">
         <v>1</v>
       </c>
       <c r="G50" t="n">
-        <v>13000</v>
+        <v>8850</v>
       </c>
       <c r="H50" t="n">
-        <v>0</v>
+        <v>885000</v>
       </c>
       <c r="I50" t="n">
         <v>0</v>
@@ -2485,7 +2457,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Lem Putih S50(E) 8 ons</t>
+          <t>GP - 5505 - HV (S = 50 EMAS) 4 ONS</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -2493,27 +2465,23 @@
           <t>Lem Putih</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>E800</t>
-        </is>
-      </c>
+      <c r="C51" t="inlineStr"/>
       <c r="D51" t="inlineStr">
         <is>
           <t>PCS</t>
         </is>
       </c>
       <c r="E51" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="F51" t="n">
         <v>1</v>
       </c>
       <c r="G51" t="n">
-        <v>16000</v>
+        <v>9900</v>
       </c>
       <c r="H51" t="n">
-        <v>0</v>
+        <v>990000</v>
       </c>
       <c r="I51" t="n">
         <v>0</v>
@@ -2526,7 +2494,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Lem Putih S50(E) 8 ons</t>
+          <t>GP - 5505 - HV (S = 50 EMAS) 6,5 ONS</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2534,27 +2502,23 @@
           <t>Lem Putih</t>
         </is>
       </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>100080</t>
-        </is>
-      </c>
+      <c r="C52" t="inlineStr"/>
       <c r="D52" t="inlineStr">
         <is>
           <t>PCS</t>
         </is>
       </c>
       <c r="E52" t="n">
-        <v>1</v>
+        <v>50</v>
       </c>
       <c r="F52" t="n">
         <v>1</v>
       </c>
       <c r="G52" t="n">
-        <v>16000</v>
+        <v>15350</v>
       </c>
       <c r="H52" t="n">
-        <v>0</v>
+        <v>767500</v>
       </c>
       <c r="I52" t="n">
         <v>0</v>
@@ -2567,35 +2531,31 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>MR LUX Botol 1/2kg</t>
+          <t>GP - 5505 - HV (S = 50 EMAS) 8 ONS</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>MR LUX Botol</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>B1/2</t>
-        </is>
-      </c>
+          <t>Lem Putih</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr"/>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Set</t>
+          <t>PCS</t>
         </is>
       </c>
       <c r="E53" t="n">
-        <v>15</v>
+        <v>50</v>
       </c>
       <c r="F53" t="n">
         <v>1</v>
       </c>
       <c r="G53" t="n">
-        <v>68000</v>
+        <v>18500</v>
       </c>
       <c r="H53" t="n">
-        <v>0</v>
+        <v>925000</v>
       </c>
       <c r="I53" t="n">
         <v>0</v>
@@ -2608,35 +2568,31 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>MR LUX Botol 1/4kg</t>
+          <t>GP - 5505 - HV (S = 50 EMAS) 2,5 Kg</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>MR LUX Botol</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>B1/4</t>
-        </is>
-      </c>
+          <t>Lem Putih</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr"/>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Set</t>
+          <t>PCS</t>
         </is>
       </c>
       <c r="E54" t="n">
-        <v>48</v>
+        <v>14</v>
       </c>
       <c r="F54" t="n">
         <v>1</v>
       </c>
       <c r="G54" t="n">
-        <v>31000</v>
+        <v>72500</v>
       </c>
       <c r="H54" t="n">
-        <v>0</v>
+        <v>1015000</v>
       </c>
       <c r="I54" t="n">
         <v>0</v>
@@ -2649,32 +2605,28 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>MR LUX Botol 1kg</t>
+          <t>GP - 5505 - HV (S = 50 EMAS) GALLON 3 KG</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>MR LUX Botol</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>B1</t>
-        </is>
-      </c>
+          <t>Lem Putih</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr"/>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Set</t>
+          <t>PCS</t>
         </is>
       </c>
       <c r="E55" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="F55" t="n">
         <v>1</v>
       </c>
       <c r="G55" t="n">
-        <v>124000</v>
+        <v>83000</v>
       </c>
       <c r="H55" t="n">
         <v>0</v>
@@ -2690,19 +2642,15 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>MR LUX Jerigen</t>
+          <t>GP - 5505 - HV (S = 50 EMAS) GALLON 3,5 KG</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>MR LUX Jerigen</t>
-        </is>
-      </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>J4KG</t>
-        </is>
-      </c>
+          <t>Lem Putih</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr"/>
       <c r="D56" t="inlineStr">
         <is>
           <t>PCS</t>
@@ -2715,7 +2663,7 @@
         <v>1</v>
       </c>
       <c r="G56" t="n">
-        <v>572000</v>
+        <v>93500</v>
       </c>
       <c r="H56" t="n">
         <v>0</v>
@@ -2731,32 +2679,28 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>MR LUX Kaleng 1/2kg</t>
+          <t>GP - 5505 - HV (S = 50 EMAS) GALLON 4 KG</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>MR LUX Kaleng</t>
-        </is>
-      </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>K1/2</t>
-        </is>
-      </c>
+          <t>Lem Putih</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr"/>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Set</t>
+          <t>PCS</t>
         </is>
       </c>
       <c r="E57" t="n">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="F57" t="n">
         <v>1</v>
       </c>
       <c r="G57" t="n">
-        <v>54000</v>
+        <v>104000</v>
       </c>
       <c r="H57" t="n">
         <v>0</v>
@@ -2772,32 +2716,28 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>MR LUX Kaleng 1/4kg</t>
+          <t>GP - 5505 - HV (S = 50 EMAS) JERIGEN 5 Kg</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>MR LUX Kaleng</t>
-        </is>
-      </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>K1/4</t>
-        </is>
-      </c>
+          <t>Lem Putih</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr"/>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Set</t>
+          <t>PCS</t>
         </is>
       </c>
       <c r="E58" t="n">
-        <v>48</v>
+        <v>1</v>
       </c>
       <c r="F58" t="n">
         <v>1</v>
       </c>
       <c r="G58" t="n">
-        <v>32000</v>
+        <v>117000</v>
       </c>
       <c r="H58" t="n">
         <v>0</v>
@@ -2813,35 +2753,31 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>MR LUX Kaleng 1kg</t>
+          <t>V - 5040 A (S = 40 MERAH) 3,5 ONS</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>MR LUX Kaleng</t>
-        </is>
-      </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>K1</t>
-        </is>
-      </c>
+          <t>Lem Putih</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr"/>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Set</t>
+          <t>PCS</t>
         </is>
       </c>
       <c r="E59" t="n">
-        <v>12</v>
+        <v>100</v>
       </c>
       <c r="F59" t="n">
         <v>1</v>
       </c>
       <c r="G59" t="n">
-        <v>107000</v>
+        <v>7800</v>
       </c>
       <c r="H59" t="n">
-        <v>0</v>
+        <v>780000</v>
       </c>
       <c r="I59" t="n">
         <v>0</v>
@@ -2854,35 +2790,31 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>MR LUX Non Sag 1 Ons</t>
+          <t>V - 5040 A (S = 40 MERAH) 4 ONS</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Non Sag</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>NS1O</t>
-        </is>
-      </c>
+          <t>Lem Putih</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr"/>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Set</t>
+          <t>PCS</t>
         </is>
       </c>
       <c r="E60" t="n">
-        <v>48</v>
+        <v>100</v>
       </c>
       <c r="F60" t="n">
         <v>1</v>
       </c>
       <c r="G60" t="n">
-        <v>25000</v>
+        <v>8700</v>
       </c>
       <c r="H60" t="n">
-        <v>0</v>
+        <v>870000</v>
       </c>
       <c r="I60" t="n">
         <v>0</v>
@@ -2895,35 +2827,31 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>MR LUX Non Sag 1 kg</t>
+          <t>V - 5040 A (S = 40 MERAH) 6,5 ONS</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Non Sag</t>
-        </is>
-      </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>NS1</t>
-        </is>
-      </c>
+          <t>Lem Putih</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr"/>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Set</t>
+          <t>PCS</t>
         </is>
       </c>
       <c r="E61" t="n">
-        <v>8</v>
+        <v>50</v>
       </c>
       <c r="F61" t="n">
         <v>1</v>
       </c>
       <c r="G61" t="n">
-        <v>175000</v>
+        <v>13500</v>
       </c>
       <c r="H61" t="n">
-        <v>0</v>
+        <v>675000</v>
       </c>
       <c r="I61" t="n">
         <v>0</v>
@@ -2936,35 +2864,31 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>MR LUX Non Sag 1/2 kg</t>
+          <t>V - 5040 A (S = 40 MERAH) 8 ONS</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Non Sag</t>
-        </is>
-      </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>NS1/2</t>
-        </is>
-      </c>
+          <t>Lem Putih</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr"/>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Set</t>
+          <t>PCS</t>
         </is>
       </c>
       <c r="E62" t="n">
-        <v>12</v>
+        <v>50</v>
       </c>
       <c r="F62" t="n">
         <v>1</v>
       </c>
       <c r="G62" t="n">
-        <v>97500</v>
+        <v>16100</v>
       </c>
       <c r="H62" t="n">
-        <v>0</v>
+        <v>805000</v>
       </c>
       <c r="I62" t="n">
         <v>0</v>
@@ -2977,35 +2901,31 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>MR LUX Non Sag 1/4 kg</t>
+          <t>P - 740 (S = 30 HITAM) 3,5 ONS</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Non Sag</t>
-        </is>
-      </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>NS1/4</t>
-        </is>
-      </c>
+          <t>Lem Putih</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr"/>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Set</t>
+          <t>PCS</t>
         </is>
       </c>
       <c r="E63" t="n">
-        <v>36</v>
+        <v>100</v>
       </c>
       <c r="F63" t="n">
         <v>1</v>
       </c>
       <c r="G63" t="n">
-        <v>48000</v>
+        <v>7400</v>
       </c>
       <c r="H63" t="n">
-        <v>0</v>
+        <v>740000</v>
       </c>
       <c r="I63" t="n">
         <v>0</v>
@@ -3018,35 +2938,31 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>NPEL 128</t>
+          <t>P - 740 (S = 30 HITAM) 4 ONS</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Umum</t>
-        </is>
-      </c>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>100020</t>
-        </is>
-      </c>
+          <t>Lem Putih</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr"/>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Drum</t>
+          <t>PCS</t>
         </is>
       </c>
       <c r="E64" t="n">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="F64" t="n">
         <v>1</v>
       </c>
       <c r="G64" t="n">
-        <v>1296000</v>
+        <v>8250</v>
       </c>
       <c r="H64" t="n">
-        <v>0</v>
+        <v>825000</v>
       </c>
       <c r="I64" t="n">
         <v>0</v>
@@ -3059,35 +2975,31 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>New B1/2 Kg  Hardener</t>
+          <t>P - 740 (S = 30 HITAM) 6,5 ONS</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Umum</t>
-        </is>
-      </c>
-      <c r="C65" t="inlineStr">
-        <is>
-          <t>NB1/2H</t>
-        </is>
-      </c>
+          <t>Lem Putih</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr"/>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Set</t>
+          <t>PCS</t>
         </is>
       </c>
       <c r="E65" t="n">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="F65" t="n">
         <v>1</v>
       </c>
       <c r="G65" t="n">
-        <v>1296000</v>
+        <v>12650</v>
       </c>
       <c r="H65" t="n">
-        <v>0</v>
+        <v>632500</v>
       </c>
       <c r="I65" t="n">
         <v>0</v>
@@ -3100,35 +3012,31 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>New MR B1Kg  Hardener</t>
+          <t>P - 740 (S = 30 HITAM) 8 ONS</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>epoxy</t>
-        </is>
-      </c>
-      <c r="C66" t="inlineStr">
-        <is>
-          <t>NB1H</t>
-        </is>
-      </c>
+          <t>Lem Putih</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr"/>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Set</t>
+          <t>PCS</t>
         </is>
       </c>
       <c r="E66" t="n">
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="F66" t="n">
         <v>1</v>
       </c>
       <c r="G66" t="n">
-        <v>1284000</v>
+        <v>15200</v>
       </c>
       <c r="H66" t="n">
-        <v>0</v>
+        <v>760000</v>
       </c>
       <c r="I66" t="n">
         <v>0</v>
@@ -3141,35 +3049,31 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>New MR Botol 1/2kg</t>
+          <t>P - 740 (S = 30 HITAM) 2,5 KG</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>New MR Botol</t>
-        </is>
-      </c>
-      <c r="C67" t="inlineStr">
-        <is>
-          <t>NB1/2</t>
-        </is>
-      </c>
+          <t>Lem Putih</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr"/>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Set</t>
+          <t>PCS</t>
         </is>
       </c>
       <c r="E67" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F67" t="n">
         <v>1</v>
       </c>
       <c r="G67" t="n">
-        <v>54000</v>
+        <v>37500</v>
       </c>
       <c r="H67" t="n">
-        <v>0</v>
+        <v>525000</v>
       </c>
       <c r="I67" t="n">
         <v>0</v>
@@ -3182,32 +3086,28 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>New MR Botol 1kg</t>
+          <t>P - 740 (S = 30 HITAM) GALLON 3 KG</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>New MR Botol</t>
-        </is>
-      </c>
-      <c r="C68" t="inlineStr">
-        <is>
-          <t>NB1</t>
-        </is>
-      </c>
+          <t>Lem Putih</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr"/>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Set</t>
+          <t>PCS</t>
         </is>
       </c>
       <c r="E68" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="F68" t="n">
         <v>1</v>
       </c>
       <c r="G68" t="n">
-        <v>107000</v>
+        <v>70500</v>
       </c>
       <c r="H68" t="n">
         <v>0</v>
@@ -3223,32 +3123,28 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>New MR Kaleng 1kg</t>
+          <t>P - 740 (S = 30 HITAM) GALLON 4 KG</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>New MR Kaleng</t>
-        </is>
-      </c>
-      <c r="C69" t="inlineStr">
-        <is>
-          <t>NK1</t>
-        </is>
-      </c>
+          <t>Lem Putih</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr"/>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Set</t>
+          <t>PCS</t>
         </is>
       </c>
       <c r="E69" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="F69" t="n">
         <v>1</v>
       </c>
       <c r="G69" t="n">
-        <v>99000</v>
+        <v>87000</v>
       </c>
       <c r="H69" t="n">
         <v>0</v>
@@ -3260,826 +3156,6 @@
         <v>0</v>
       </c>
       <c r="K69" t="inlineStr"/>
-    </row>
-    <row r="70">
-      <c r="A70" t="inlineStr">
-        <is>
-          <t>PU 1 P</t>
-        </is>
-      </c>
-      <c r="B70" t="inlineStr">
-        <is>
-          <t>PU</t>
-        </is>
-      </c>
-      <c r="C70" t="inlineStr">
-        <is>
-          <t>100015</t>
-        </is>
-      </c>
-      <c r="D70" t="inlineStr">
-        <is>
-          <t>PCS</t>
-        </is>
-      </c>
-      <c r="E70" t="n">
-        <v>1</v>
-      </c>
-      <c r="F70" t="n">
-        <v>1</v>
-      </c>
-      <c r="G70" t="n">
-        <v>121000</v>
-      </c>
-      <c r="H70" t="n">
-        <v>0</v>
-      </c>
-      <c r="I70" t="n">
-        <v>0</v>
-      </c>
-      <c r="J70" t="n">
-        <v>0</v>
-      </c>
-      <c r="K70" t="inlineStr"/>
-    </row>
-    <row r="71">
-      <c r="A71" t="inlineStr">
-        <is>
-          <t>PU 1/2 P</t>
-        </is>
-      </c>
-      <c r="B71" t="inlineStr">
-        <is>
-          <t>PU</t>
-        </is>
-      </c>
-      <c r="C71" t="inlineStr">
-        <is>
-          <t>100016</t>
-        </is>
-      </c>
-      <c r="D71" t="inlineStr">
-        <is>
-          <t>PCS</t>
-        </is>
-      </c>
-      <c r="E71" t="n">
-        <v>1</v>
-      </c>
-      <c r="F71" t="n">
-        <v>1</v>
-      </c>
-      <c r="G71" t="n">
-        <v>1296000</v>
-      </c>
-      <c r="H71" t="n">
-        <v>0</v>
-      </c>
-      <c r="I71" t="n">
-        <v>0</v>
-      </c>
-      <c r="J71" t="n">
-        <v>0</v>
-      </c>
-      <c r="K71" t="inlineStr"/>
-    </row>
-    <row r="72">
-      <c r="A72" t="inlineStr">
-        <is>
-          <t>PU 1/2 Putih</t>
-        </is>
-      </c>
-      <c r="B72" t="inlineStr">
-        <is>
-          <t>PU</t>
-        </is>
-      </c>
-      <c r="C72" t="inlineStr">
-        <is>
-          <t>100072</t>
-        </is>
-      </c>
-      <c r="D72" t="inlineStr">
-        <is>
-          <t>Set</t>
-        </is>
-      </c>
-      <c r="E72" t="n">
-        <v>30</v>
-      </c>
-      <c r="F72" t="n">
-        <v>1</v>
-      </c>
-      <c r="G72" t="n">
-        <v>24250</v>
-      </c>
-      <c r="H72" t="n">
-        <v>0</v>
-      </c>
-      <c r="I72" t="n">
-        <v>0</v>
-      </c>
-      <c r="J72" t="n">
-        <v>0</v>
-      </c>
-      <c r="K72" t="inlineStr"/>
-    </row>
-    <row r="73">
-      <c r="A73" t="inlineStr">
-        <is>
-          <t>PU 1/2 kg MR LUX</t>
-        </is>
-      </c>
-      <c r="B73" t="inlineStr">
-        <is>
-          <t>PU</t>
-        </is>
-      </c>
-      <c r="C73" t="inlineStr">
-        <is>
-          <t>PU1/2</t>
-        </is>
-      </c>
-      <c r="D73" t="inlineStr">
-        <is>
-          <t>PCS</t>
-        </is>
-      </c>
-      <c r="E73" t="n">
-        <v>30</v>
-      </c>
-      <c r="F73" t="n">
-        <v>1</v>
-      </c>
-      <c r="G73" t="n">
-        <v>34500</v>
-      </c>
-      <c r="H73" t="n">
-        <v>0</v>
-      </c>
-      <c r="I73" t="n">
-        <v>0</v>
-      </c>
-      <c r="J73" t="n">
-        <v>0</v>
-      </c>
-      <c r="K73" t="inlineStr"/>
-    </row>
-    <row r="74">
-      <c r="A74" t="inlineStr">
-        <is>
-          <t>PU 1/2kg WoodLux</t>
-        </is>
-      </c>
-      <c r="B74" t="inlineStr">
-        <is>
-          <t>Wood Lux</t>
-        </is>
-      </c>
-      <c r="C74" t="inlineStr">
-        <is>
-          <t>WL1/2</t>
-        </is>
-      </c>
-      <c r="D74" t="inlineStr">
-        <is>
-          <t>PCS</t>
-        </is>
-      </c>
-      <c r="E74" t="n">
-        <v>30</v>
-      </c>
-      <c r="F74" t="n">
-        <v>1</v>
-      </c>
-      <c r="G74" t="n">
-        <v>27000</v>
-      </c>
-      <c r="H74" t="n">
-        <v>0</v>
-      </c>
-      <c r="I74" t="n">
-        <v>0</v>
-      </c>
-      <c r="J74" t="n">
-        <v>0</v>
-      </c>
-      <c r="K74" t="inlineStr"/>
-    </row>
-    <row r="75">
-      <c r="A75" t="inlineStr">
-        <is>
-          <t>PU 1/4kg MR LUX</t>
-        </is>
-      </c>
-      <c r="B75" t="inlineStr">
-        <is>
-          <t>PU</t>
-        </is>
-      </c>
-      <c r="C75" t="inlineStr">
-        <is>
-          <t>PU1/4</t>
-        </is>
-      </c>
-      <c r="D75" t="inlineStr">
-        <is>
-          <t>PCS</t>
-        </is>
-      </c>
-      <c r="E75" t="n">
-        <v>95</v>
-      </c>
-      <c r="F75" t="n">
-        <v>1</v>
-      </c>
-      <c r="G75" t="n">
-        <v>17000</v>
-      </c>
-      <c r="H75" t="n">
-        <v>0</v>
-      </c>
-      <c r="I75" t="n">
-        <v>0</v>
-      </c>
-      <c r="J75" t="n">
-        <v>0</v>
-      </c>
-      <c r="K75" t="inlineStr"/>
-    </row>
-    <row r="76">
-      <c r="A76" t="inlineStr">
-        <is>
-          <t>PU 1kg MR LUX</t>
-        </is>
-      </c>
-      <c r="B76" t="inlineStr">
-        <is>
-          <t>PU</t>
-        </is>
-      </c>
-      <c r="C76" t="inlineStr">
-        <is>
-          <t>PU1</t>
-        </is>
-      </c>
-      <c r="D76" t="inlineStr">
-        <is>
-          <t>PCS</t>
-        </is>
-      </c>
-      <c r="E76" t="n">
-        <v>20</v>
-      </c>
-      <c r="F76" t="n">
-        <v>1</v>
-      </c>
-      <c r="G76" t="n">
-        <v>67000</v>
-      </c>
-      <c r="H76" t="n">
-        <v>0</v>
-      </c>
-      <c r="I76" t="n">
-        <v>0</v>
-      </c>
-      <c r="J76" t="n">
-        <v>0</v>
-      </c>
-      <c r="K76" t="inlineStr"/>
-    </row>
-    <row r="77">
-      <c r="A77" t="inlineStr">
-        <is>
-          <t>PU 1kg WoodLux</t>
-        </is>
-      </c>
-      <c r="B77" t="inlineStr">
-        <is>
-          <t>Wood Lux</t>
-        </is>
-      </c>
-      <c r="C77" t="inlineStr">
-        <is>
-          <t>WL1</t>
-        </is>
-      </c>
-      <c r="D77" t="inlineStr">
-        <is>
-          <t>PCS</t>
-        </is>
-      </c>
-      <c r="E77" t="n">
-        <v>20</v>
-      </c>
-      <c r="F77" t="n">
-        <v>1</v>
-      </c>
-      <c r="G77" t="n">
-        <v>57000</v>
-      </c>
-      <c r="H77" t="n">
-        <v>0</v>
-      </c>
-      <c r="I77" t="n">
-        <v>0</v>
-      </c>
-      <c r="J77" t="n">
-        <v>0</v>
-      </c>
-      <c r="K77" t="inlineStr"/>
-    </row>
-    <row r="78">
-      <c r="A78" t="inlineStr">
-        <is>
-          <t>Pengiriman</t>
-        </is>
-      </c>
-      <c r="B78" t="inlineStr">
-        <is>
-          <t>epoxy</t>
-        </is>
-      </c>
-      <c r="C78" t="inlineStr">
-        <is>
-          <t>100083</t>
-        </is>
-      </c>
-      <c r="D78" t="inlineStr">
-        <is>
-          <t>PCS</t>
-        </is>
-      </c>
-      <c r="E78" t="n">
-        <v>1</v>
-      </c>
-      <c r="F78" t="n">
-        <v>1</v>
-      </c>
-      <c r="G78" t="n">
-        <v>0</v>
-      </c>
-      <c r="H78" t="n">
-        <v>0</v>
-      </c>
-      <c r="I78" t="n">
-        <v>0</v>
-      </c>
-      <c r="J78" t="n">
-        <v>0</v>
-      </c>
-      <c r="K78" t="inlineStr"/>
-    </row>
-    <row r="79">
-      <c r="A79" t="inlineStr">
-        <is>
-          <t>RESIN NPEL</t>
-        </is>
-      </c>
-      <c r="B79" t="inlineStr">
-        <is>
-          <t>DRUM</t>
-        </is>
-      </c>
-      <c r="C79" t="inlineStr">
-        <is>
-          <t>100074</t>
-        </is>
-      </c>
-      <c r="D79" t="inlineStr">
-        <is>
-          <t>Drum</t>
-        </is>
-      </c>
-      <c r="E79" t="n">
-        <v>1</v>
-      </c>
-      <c r="F79" t="n">
-        <v>1</v>
-      </c>
-      <c r="G79" t="n">
-        <v>0</v>
-      </c>
-      <c r="H79" t="n">
-        <v>0</v>
-      </c>
-      <c r="I79" t="n">
-        <v>0</v>
-      </c>
-      <c r="J79" t="n">
-        <v>0</v>
-      </c>
-      <c r="K79" t="inlineStr"/>
-    </row>
-    <row r="80">
-      <c r="A80" t="inlineStr">
-        <is>
-          <t>Resin</t>
-        </is>
-      </c>
-      <c r="B80" t="inlineStr">
-        <is>
-          <t>Umum</t>
-        </is>
-      </c>
-      <c r="C80" t="inlineStr">
-        <is>
-          <t>100042</t>
-        </is>
-      </c>
-      <c r="D80" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="E80" t="n">
-        <v>1</v>
-      </c>
-      <c r="F80" t="n">
-        <v>1</v>
-      </c>
-      <c r="G80" t="n">
-        <v>0</v>
-      </c>
-      <c r="H80" t="n">
-        <v>0</v>
-      </c>
-      <c r="I80" t="n">
-        <v>0</v>
-      </c>
-      <c r="J80" t="n">
-        <v>0</v>
-      </c>
-      <c r="K80" t="inlineStr"/>
-    </row>
-    <row r="81">
-      <c r="A81" t="inlineStr">
-        <is>
-          <t>S30 Lem Putih (2,5 kg)</t>
-        </is>
-      </c>
-      <c r="B81" t="inlineStr">
-        <is>
-          <t>Lem Putih</t>
-        </is>
-      </c>
-      <c r="C81" t="inlineStr">
-        <is>
-          <t>100041</t>
-        </is>
-      </c>
-      <c r="D81" t="inlineStr">
-        <is>
-          <t>PCS</t>
-        </is>
-      </c>
-      <c r="E81" t="n">
-        <v>1</v>
-      </c>
-      <c r="F81" t="n">
-        <v>1</v>
-      </c>
-      <c r="G81" t="n">
-        <v>39000</v>
-      </c>
-      <c r="H81" t="n">
-        <v>0</v>
-      </c>
-      <c r="I81" t="n">
-        <v>0</v>
-      </c>
-      <c r="J81" t="n">
-        <v>0</v>
-      </c>
-      <c r="K81" t="inlineStr"/>
-    </row>
-    <row r="82">
-      <c r="A82" t="inlineStr">
-        <is>
-          <t>S30 Lem Putih (3,5 ons)</t>
-        </is>
-      </c>
-      <c r="B82" t="inlineStr">
-        <is>
-          <t>Lem Putih</t>
-        </is>
-      </c>
-      <c r="C82" t="inlineStr">
-        <is>
-          <t>100037</t>
-        </is>
-      </c>
-      <c r="D82" t="inlineStr">
-        <is>
-          <t>PCS</t>
-        </is>
-      </c>
-      <c r="E82" t="n">
-        <v>1</v>
-      </c>
-      <c r="F82" t="n">
-        <v>1</v>
-      </c>
-      <c r="G82" t="n">
-        <v>6250</v>
-      </c>
-      <c r="H82" t="n">
-        <v>0</v>
-      </c>
-      <c r="I82" t="n">
-        <v>0</v>
-      </c>
-      <c r="J82" t="n">
-        <v>0</v>
-      </c>
-      <c r="K82" t="inlineStr"/>
-    </row>
-    <row r="83">
-      <c r="A83" t="inlineStr">
-        <is>
-          <t>S30 Lem Putih (4 ons)</t>
-        </is>
-      </c>
-      <c r="B83" t="inlineStr">
-        <is>
-          <t>Lem Putih</t>
-        </is>
-      </c>
-      <c r="C83" t="inlineStr">
-        <is>
-          <t>100038</t>
-        </is>
-      </c>
-      <c r="D83" t="inlineStr">
-        <is>
-          <t>PCS</t>
-        </is>
-      </c>
-      <c r="E83" t="n">
-        <v>1</v>
-      </c>
-      <c r="F83" t="n">
-        <v>1</v>
-      </c>
-      <c r="G83" t="n">
-        <v>7000</v>
-      </c>
-      <c r="H83" t="n">
-        <v>0</v>
-      </c>
-      <c r="I83" t="n">
-        <v>0</v>
-      </c>
-      <c r="J83" t="n">
-        <v>0</v>
-      </c>
-      <c r="K83" t="inlineStr"/>
-    </row>
-    <row r="84">
-      <c r="A84" t="inlineStr">
-        <is>
-          <t>S30 Lem Putih (8 ons)</t>
-        </is>
-      </c>
-      <c r="B84" t="inlineStr">
-        <is>
-          <t>Lem Putih</t>
-        </is>
-      </c>
-      <c r="C84" t="inlineStr">
-        <is>
-          <t>100040</t>
-        </is>
-      </c>
-      <c r="D84" t="inlineStr">
-        <is>
-          <t>PCS</t>
-        </is>
-      </c>
-      <c r="E84" t="n">
-        <v>1</v>
-      </c>
-      <c r="F84" t="n">
-        <v>1</v>
-      </c>
-      <c r="G84" t="n">
-        <v>13000</v>
-      </c>
-      <c r="H84" t="n">
-        <v>0</v>
-      </c>
-      <c r="I84" t="n">
-        <v>0</v>
-      </c>
-      <c r="J84" t="n">
-        <v>0</v>
-      </c>
-      <c r="K84" t="inlineStr"/>
-    </row>
-    <row r="85">
-      <c r="A85" t="inlineStr">
-        <is>
-          <t>S40 Lem Putih (2,5 kg)</t>
-        </is>
-      </c>
-      <c r="B85" t="inlineStr">
-        <is>
-          <t>Lem Putih</t>
-        </is>
-      </c>
-      <c r="C85" t="inlineStr">
-        <is>
-          <t>100035</t>
-        </is>
-      </c>
-      <c r="D85" t="inlineStr">
-        <is>
-          <t>PCS</t>
-        </is>
-      </c>
-      <c r="E85" t="n">
-        <v>1</v>
-      </c>
-      <c r="F85" t="n">
-        <v>1</v>
-      </c>
-      <c r="G85" t="n">
-        <v>55000</v>
-      </c>
-      <c r="H85" t="n">
-        <v>0</v>
-      </c>
-      <c r="I85" t="n">
-        <v>0</v>
-      </c>
-      <c r="J85" t="n">
-        <v>0</v>
-      </c>
-      <c r="K85" t="inlineStr"/>
-    </row>
-    <row r="86">
-      <c r="A86" t="inlineStr">
-        <is>
-          <t>S40 Lem Putih (3,5 ons)</t>
-        </is>
-      </c>
-      <c r="B86" t="inlineStr">
-        <is>
-          <t>Lem Putih</t>
-        </is>
-      </c>
-      <c r="C86" t="inlineStr">
-        <is>
-          <t>100031</t>
-        </is>
-      </c>
-      <c r="D86" t="inlineStr">
-        <is>
-          <t>PCS</t>
-        </is>
-      </c>
-      <c r="E86" t="n">
-        <v>1</v>
-      </c>
-      <c r="F86" t="n">
-        <v>1</v>
-      </c>
-      <c r="G86" t="n">
-        <v>8350</v>
-      </c>
-      <c r="H86" t="n">
-        <v>0</v>
-      </c>
-      <c r="I86" t="n">
-        <v>0</v>
-      </c>
-      <c r="J86" t="n">
-        <v>0</v>
-      </c>
-      <c r="K86" t="inlineStr"/>
-    </row>
-    <row r="87">
-      <c r="A87" t="inlineStr">
-        <is>
-          <t>S40 Lem Putih (3kg)</t>
-        </is>
-      </c>
-      <c r="B87" t="inlineStr">
-        <is>
-          <t>Lem Putih</t>
-        </is>
-      </c>
-      <c r="C87" t="inlineStr">
-        <is>
-          <t>100036</t>
-        </is>
-      </c>
-      <c r="D87" t="inlineStr">
-        <is>
-          <t>PCS</t>
-        </is>
-      </c>
-      <c r="E87" t="n">
-        <v>1</v>
-      </c>
-      <c r="F87" t="n">
-        <v>1</v>
-      </c>
-      <c r="G87" t="n">
-        <v>114000</v>
-      </c>
-      <c r="H87" t="n">
-        <v>0</v>
-      </c>
-      <c r="I87" t="n">
-        <v>0</v>
-      </c>
-      <c r="J87" t="n">
-        <v>0</v>
-      </c>
-      <c r="K87" t="inlineStr"/>
-    </row>
-    <row r="88">
-      <c r="A88" t="inlineStr">
-        <is>
-          <t>S40 Lem Putih (4 ons)</t>
-        </is>
-      </c>
-      <c r="B88" t="inlineStr">
-        <is>
-          <t>Lem Putih</t>
-        </is>
-      </c>
-      <c r="C88" t="inlineStr">
-        <is>
-          <t>100032</t>
-        </is>
-      </c>
-      <c r="D88" t="inlineStr">
-        <is>
-          <t>PCS</t>
-        </is>
-      </c>
-      <c r="E88" t="n">
-        <v>1</v>
-      </c>
-      <c r="F88" t="n">
-        <v>1</v>
-      </c>
-      <c r="G88" t="n">
-        <v>9400</v>
-      </c>
-      <c r="H88" t="n">
-        <v>0</v>
-      </c>
-      <c r="I88" t="n">
-        <v>0</v>
-      </c>
-      <c r="J88" t="n">
-        <v>0</v>
-      </c>
-      <c r="K88" t="inlineStr"/>
-    </row>
-    <row r="89">
-      <c r="A89" t="inlineStr">
-        <is>
-          <t>S40 Lem Putih (8 ons)</t>
-        </is>
-      </c>
-      <c r="B89" t="inlineStr">
-        <is>
-          <t>Lem Putih</t>
-        </is>
-      </c>
-      <c r="C89" t="inlineStr">
-        <is>
-          <t>100034</t>
-        </is>
-      </c>
-      <c r="D89" t="inlineStr">
-        <is>
-          <t>PCS</t>
-        </is>
-      </c>
-      <c r="E89" t="n">
-        <v>1</v>
-      </c>
-      <c r="F89" t="n">
-        <v>1</v>
-      </c>
-      <c r="G89" t="n">
-        <v>17800</v>
-      </c>
-      <c r="H89" t="n">
-        <v>0</v>
-      </c>
-      <c r="I89" t="n">
-        <v>0</v>
-      </c>
-      <c r="J89" t="n">
-        <v>0</v>
-      </c>
-      <c r="K89" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>